<commit_message>
fix: make the bulk-import template's example row unmistakably a placeholder
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/student-bulk-import-template.xlsx
+++ b/apps/web/public/templates/student-bulk-import-template.xlsx
@@ -79,10 +79,10 @@
     <t>Parent 2 Primary Contact (Yes/No)</t>
   </si>
   <si>
-    <t>Ada</t>
-  </si>
-  <si>
-    <t>Bello</t>
+    <t>EXAMPLE</t>
+  </si>
+  <si>
+    <t>DELETE-THIS-ROW</t>
   </si>
   <si>
     <t/>
@@ -94,13 +94,13 @@
     <t>Female</t>
   </si>
   <si>
-    <t>Chidi</t>
-  </si>
-  <si>
-    <t>chidi.bello@example.com</t>
-  </si>
-  <si>
-    <t>Father</t>
+    <t>PARENT-DELETE-THIS-ROW</t>
+  </si>
+  <si>
+    <t>delete-this-example-row@example.com</t>
+  </si>
+  <si>
+    <t>Mother</t>
   </si>
   <si>
     <t>Yes</t>
@@ -514,7 +514,7 @@
     <col min="22" max="22" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -614,10 +614,10 @@
         <v>24</v>
       </c>
       <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
         <v>27</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
       </c>
       <c r="M2" t="s">
         <v>28</v>

</xml_diff>